<commit_message>
support for automatic calculation of control rows (ZakupCtrl / SprzedazCtrl)
</commit_message>
<xml_diff>
--- a/przykladowe-pliki-wejsciowe/przyklad-sekcje.xlsx
+++ b/przykladowe-pliki-wejsciowe/przyklad-sekcje.xlsx
@@ -186,7 +186,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="87">
   <si>
     <t xml:space="preserve">SEKCJA</t>
   </si>
@@ -359,6 +359,12 @@
     <t xml:space="preserve">K_20</t>
   </si>
   <si>
+    <t xml:space="preserve">K_35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TypDokumentu</t>
+  </si>
+  <si>
     <t xml:space="preserve">NAZWA 1</t>
   </si>
   <si>
@@ -368,16 +374,19 @@
     <t xml:space="preserve">2020-09-01</t>
   </si>
   <si>
-    <t xml:space="preserve">SPRZEDAZ-CTRL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LiczbaWierszySprzedazy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PodatekNalezny</t>
-  </si>
-  <si>
-    <t xml:space="preserve">55.66</t>
+    <t xml:space="preserve">15.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAZWA 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">222/333/45444</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-09-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP</t>
   </si>
   <si>
     <t xml:space="preserve">ZAKUP</t>
@@ -434,27 +443,22 @@
     <t xml:space="preserve">2020-08-31</t>
   </si>
   <si>
-    <t xml:space="preserve">ZAKUP-CTRL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LiczbaWierszyZakupow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PodatekNaliczony</t>
-  </si>
-  <si>
-    <t xml:space="preserve">111.22</t>
+    <t xml:space="preserve">148.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.33</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -491,12 +495,27 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -518,19 +537,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF81D41A"/>
-        <bgColor rgb="FFAFD095"/>
+        <bgColor rgb="FF969696"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF3465A4"/>
         <bgColor rgb="FF3366FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFAFD095"/>
-        <bgColor rgb="FF99CCFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -543,12 +556,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF8000"/>
         <bgColor rgb="FFFF7B59"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF50938A"/>
-        <bgColor rgb="FF808080"/>
       </patternFill>
     </fill>
   </fills>
@@ -586,7 +593,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -619,18 +626,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -639,47 +634,47 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -708,7 +703,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFAFD095"/>
+      <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -743,7 +738,7 @@
       <rgbColor rgb="FF3465A4"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF50938A"/>
+      <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
@@ -866,11 +861,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BN36"/>
+  <dimension ref="A1:BN1048576"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="14.65" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.67"/>
@@ -879,7 +874,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="5.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="61" min="11" style="1" width="10.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="11" style="1" width="10.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="13.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="61" min="25" style="1" width="10.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="62" min="62" style="1" width="12.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="63" min="63" style="1" width="18.34"/>
   </cols>
@@ -928,11 +925,6 @@
       <c r="E3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -950,11 +942,6 @@
       <c r="E4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E5" s="4"/>
@@ -994,7 +981,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1077,40 +1064,39 @@
       <c r="BG13" s="3"/>
       <c r="BH13" s="3"/>
       <c r="BI13" s="3"/>
-      <c r="BJ13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="J14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="K14" s="7" t="s">
         <v>28</v>
       </c>
       <c r="L14" s="7" t="s">
@@ -1128,20 +1114,18 @@
       <c r="P14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="11"/>
-      <c r="W14" s="11"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
       <c r="AB14" s="3"/>
       <c r="AC14" s="3"/>
-      <c r="AD14" s="11"/>
+      <c r="AD14" s="8"/>
       <c r="AE14" s="3"/>
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
@@ -1240,37 +1224,36 @@
       <c r="BG15" s="3"/>
       <c r="BH15" s="3"/>
       <c r="BI15" s="3"/>
-      <c r="BJ15" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="12"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="12"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="12"/>
-      <c r="U18" s="12"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="9"/>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
+      <c r="S18" s="9"/>
+      <c r="T18" s="9"/>
+      <c r="U18" s="9"/>
+      <c r="V18" s="9"/>
+      <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
@@ -1310,35 +1293,35 @@
       <c r="BI18" s="3"/>
       <c r="BJ18" s="3"/>
       <c r="BK18" s="3"/>
-      <c r="BL18" s="10"/>
-      <c r="BM18" s="10"/>
-      <c r="BN18" s="10"/>
+      <c r="BL18" s="1"/>
+      <c r="BM18" s="1"/>
+      <c r="BN18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="12"/>
-      <c r="N19" s="12"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="12"/>
-      <c r="Q19" s="12"/>
-      <c r="R19" s="12"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="12"/>
-      <c r="U19" s="12"/>
-      <c r="V19" s="12"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
+      <c r="S19" s="9"/>
+      <c r="T19" s="9"/>
+      <c r="U19" s="9"/>
+      <c r="V19" s="9"/>
+      <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
       <c r="AA19" s="3"/>
@@ -1378,159 +1361,144 @@
       <c r="BI19" s="3"/>
       <c r="BJ19" s="3"/>
       <c r="BK19" s="3"/>
-      <c r="BL19" s="10"/>
-      <c r="BM19" s="10"/>
-      <c r="BN19" s="10"/>
+      <c r="BL19" s="1"/>
+      <c r="BM19" s="1"/>
+      <c r="BN19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="F20" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="H20" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="I20" s="14" t="s">
+      <c r="I20" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="J20" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="K20" s="14" t="s">
+      <c r="K20" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="L20" s="12" t="s">
+      <c r="L20" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="M20" s="12" t="s">
+      <c r="M20" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="N20" s="12" t="s">
+      <c r="N20" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="O20" s="12" t="s">
+      <c r="O20" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="P20" s="12" t="s">
+      <c r="P20" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="Q20" s="13" t="s">
+      <c r="Q20" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="R20" s="13" t="s">
+      <c r="R20" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="S20" s="13" t="s">
+      <c r="S20" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="T20" s="13" t="s">
+      <c r="T20" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="U20" s="13" t="s">
+      <c r="U20" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="V20" s="13" t="s">
+      <c r="V20" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="W20" s="3"/>
-      <c r="X20" s="3"/>
-      <c r="Y20" s="11"/>
-      <c r="Z20" s="11"/>
-      <c r="AA20" s="11"/>
-      <c r="AB20" s="11"/>
-      <c r="AC20" s="11"/>
-      <c r="AD20" s="11"/>
-      <c r="AE20" s="11"/>
-      <c r="AF20" s="11"/>
-      <c r="AG20" s="11"/>
-      <c r="AH20" s="11"/>
+      <c r="W20" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="X20" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y20" s="8"/>
+      <c r="Z20" s="8"/>
+      <c r="AA20" s="8"/>
+      <c r="AB20" s="8"/>
+      <c r="AC20" s="8"/>
+      <c r="AD20" s="8"/>
+      <c r="AE20" s="8"/>
+      <c r="AF20" s="8"/>
+      <c r="AG20" s="8"/>
+      <c r="AH20" s="8"/>
       <c r="AI20" s="3"/>
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
       <c r="AL20" s="3"/>
       <c r="AM20" s="3"/>
       <c r="AN20" s="3"/>
-      <c r="AO20" s="10"/>
-      <c r="AP20" s="10"/>
-      <c r="AQ20" s="10"/>
-      <c r="AR20" s="10"/>
-      <c r="AS20" s="10"/>
-      <c r="AT20" s="10"/>
-      <c r="AU20" s="10"/>
-      <c r="AV20" s="10"/>
-      <c r="AW20" s="10"/>
-      <c r="AX20" s="10"/>
-      <c r="AY20" s="10"/>
-      <c r="AZ20" s="10"/>
-      <c r="BA20" s="10"/>
-      <c r="BB20" s="10"/>
-      <c r="BC20" s="10"/>
-      <c r="BD20" s="10"/>
-      <c r="BE20" s="10"/>
-      <c r="BF20" s="10"/>
-      <c r="BG20" s="10"/>
-      <c r="BH20" s="10"/>
-      <c r="BI20" s="10"/>
-      <c r="BJ20" s="10"/>
-      <c r="BK20" s="10"/>
-      <c r="BL20" s="10"/>
-      <c r="BM20" s="10"/>
-      <c r="BN20" s="10"/>
+      <c r="BL20" s="1"/>
+      <c r="BM20" s="1"/>
+      <c r="BN20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="n">
+      <c r="A21" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12" t="n">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9" t="n">
         <v>11111</v>
       </c>
-      <c r="D21" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="F21" s="15" t="s">
+      <c r="D21" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="H21" s="12"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="12"/>
-      <c r="N21" s="12"/>
-      <c r="O21" s="12"/>
-      <c r="P21" s="12"/>
-      <c r="Q21" s="12"/>
-      <c r="R21" s="12"/>
-      <c r="S21" s="12"/>
-      <c r="T21" s="12"/>
-      <c r="U21" s="12"/>
-      <c r="V21" s="12"/>
-      <c r="W21" s="3"/>
-      <c r="X21" s="3"/>
+      <c r="E21" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="W21" s="9" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="X21" s="9"/>
       <c r="Y21" s="3"/>
       <c r="Z21" s="3"/>
       <c r="AA21" s="3"/>
@@ -1574,212 +1542,205 @@
       <c r="BM21" s="3"/>
       <c r="BN21" s="3"/>
     </row>
-    <row r="23" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="s">
+    <row r="22" customFormat="false" ht="14.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14" t="n">
+        <v>22222</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="14"/>
+      <c r="Q22" s="14"/>
+      <c r="R22" s="14"/>
+      <c r="S22" s="14"/>
+      <c r="T22" s="14"/>
+      <c r="U22" s="14"/>
+      <c r="V22" s="14"/>
+      <c r="W22" s="15"/>
+      <c r="X22" s="14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
+      <c r="B24" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="16"/>
+      <c r="T24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="16"/>
+      <c r="T25" s="17"/>
+    </row>
+    <row r="26" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="H26" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="J26" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="K26" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="L26" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="M26" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="N26" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="O26" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="P26" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q26" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="R26" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="S26" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="T26" s="19" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16" t="n">
+        <v>1111111</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E27" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="G27" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="16" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B28" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="17"/>
-      <c r="M28" s="17"/>
-      <c r="N28" s="17"/>
-      <c r="O28" s="17"/>
-      <c r="P28" s="17"/>
-      <c r="Q28" s="17"/>
-      <c r="R28" s="17"/>
-      <c r="S28" s="17"/>
-      <c r="T28" s="18"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="17"/>
-      <c r="M29" s="17"/>
-      <c r="N29" s="17"/>
-      <c r="O29" s="17"/>
-      <c r="P29" s="17"/>
-      <c r="Q29" s="17"/>
-      <c r="R29" s="17"/>
-      <c r="S29" s="17"/>
-      <c r="T29" s="18"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="E30" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="F30" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="H30" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="I30" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="J30" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="K30" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="L30" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="M30" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="N30" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="O30" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="P30" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q30" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="R30" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="S30" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="T30" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="U30" s="0"/>
-      <c r="V30" s="0"/>
-      <c r="BK30" s="0"/>
-    </row>
-    <row r="31" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17" t="n">
-        <v>1111111</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="F31" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="G31" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
-      <c r="P31" s="17"/>
-      <c r="Q31" s="17"/>
-      <c r="R31" s="17"/>
-      <c r="S31" s="17"/>
-      <c r="T31" s="17"/>
-      <c r="U31" s="3"/>
-      <c r="V31" s="3"/>
-      <c r="W31" s="3"/>
-    </row>
-    <row r="33" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23"/>
-      <c r="B34" s="23"/>
-    </row>
-    <row r="35" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="B35" s="23" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B36" s="23" t="s">
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16" t="s">
         <v>85</v>
       </c>
-    </row>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="16"/>
+      <c r="T27" s="16"/>
+      <c r="U27" s="3"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="3"/>
+    </row>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D10" r:id="rId2" display="firma@firma.abc.pl"/>

</xml_diff>